<commit_message>
time plots weighted by incidence
</commit_message>
<xml_diff>
--- a/markers_table.xlsx
+++ b/markers_table.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10921"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11003"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lharrison/Desktop/MARCSE/k13_seafrica/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD200CDE-47FA-AD46-933D-C624881CF89A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F24A60CC-0277-AC4F-8BE9-B1D79A2DEF70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="140" yWindow="820" windowWidth="16720" windowHeight="17240" xr2:uid="{E77422C1-C186-CE4B-A2C5-30646380C87E}"/>
+    <workbookView xWindow="140" yWindow="820" windowWidth="16720" windowHeight="17240" activeTab="1" xr2:uid="{E77422C1-C186-CE4B-A2C5-30646380C87E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="39">
   <si>
     <t>Kelch 13</t>
   </si>
@@ -128,6 +129,30 @@
   </si>
   <si>
     <t>Okell also compare to national treatment policies.</t>
+  </si>
+  <si>
+    <t>Lumefantrine</t>
+  </si>
+  <si>
+    <t>Monotherapy for Pf until resistance emerged in the 1980s? 1990s?; still used in Ethiopia to treat Pv, including where Pf and Pv co-circulate</t>
+  </si>
+  <si>
+    <t>Artemisinin (derivatives)</t>
+  </si>
+  <si>
+    <t>Sulfadoxine pyrimethamine</t>
+  </si>
+  <si>
+    <t>Chloroquine (CQ)</t>
+  </si>
+  <si>
+    <t>Amodiaquine (AQ)</t>
+  </si>
+  <si>
+    <t>Piperaquine (PPQ)</t>
+  </si>
+  <si>
+    <t>Combination therapy that replaced CQ as recommended first-line treatment</t>
   </si>
 </sst>
 </file>
@@ -621,4 +646,53 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6821B724-4309-7B42-8551-18F57DE4ECC6}">
+  <dimension ref="A2:B7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="16.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>34</v>
+      </c>
+      <c r="B7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
separated moldm and marcse tidying so that merging script is only merging
</commit_message>
<xml_diff>
--- a/markers_table.xlsx
+++ b/markers_table.xlsx
@@ -1,20 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11003"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10110"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lharrison/Desktop/MARCSE/k13_seafrica/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F24A60CC-0277-AC4F-8BE9-B1D79A2DEF70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19F08B2C-573D-A643-9004-9D8502F5F54B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="140" yWindow="820" windowWidth="16720" windowHeight="17240" activeTab="1" xr2:uid="{E77422C1-C186-CE4B-A2C5-30646380C87E}"/>
+    <workbookView xWindow="10440" yWindow="800" windowWidth="22860" windowHeight="17240" activeTab="3" xr2:uid="{E77422C1-C186-CE4B-A2C5-30646380C87E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet name="Sheet4" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -36,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="78">
   <si>
     <t>Kelch 13</t>
   </si>
@@ -153,13 +155,130 @@
   </si>
   <si>
     <t>Combination therapy that replaced CQ as recommended first-line treatment</t>
+  </si>
+  <si>
+    <t>F446I</t>
+  </si>
+  <si>
+    <t>N458Y</t>
+  </si>
+  <si>
+    <t>C469Y</t>
+  </si>
+  <si>
+    <t>M476I</t>
+  </si>
+  <si>
+    <t>Y493H</t>
+  </si>
+  <si>
+    <t>G533S</t>
+  </si>
+  <si>
+    <t>R539T</t>
+  </si>
+  <si>
+    <t>I543T</t>
+  </si>
+  <si>
+    <t>P553L</t>
+  </si>
+  <si>
+    <t>R561H</t>
+  </si>
+  <si>
+    <t>P574L</t>
+  </si>
+  <si>
+    <t>C580Y</t>
+  </si>
+  <si>
+    <t>R622I</t>
+  </si>
+  <si>
+    <t>A675V</t>
+  </si>
+  <si>
+    <t>E252Q</t>
+  </si>
+  <si>
+    <t>P441L</t>
+  </si>
+  <si>
+    <t>C469F</t>
+  </si>
+  <si>
+    <t>N537I</t>
+  </si>
+  <si>
+    <t>G538V</t>
+  </si>
+  <si>
+    <t>V568G</t>
+  </si>
+  <si>
+    <t>Validated marker (Epi., Lab. &amp; Clin.)</t>
+  </si>
+  <si>
+    <t>Candidate marker (Epi. &amp; Clin.)</t>
+  </si>
+  <si>
+    <t>WHO validated</t>
+  </si>
+  <si>
+    <t>WHO candidate</t>
+  </si>
+  <si>
+    <t>P413A</t>
+  </si>
+  <si>
+    <t>F495L</t>
+  </si>
+  <si>
+    <t>R515K</t>
+  </si>
+  <si>
+    <t>M579I</t>
+  </si>
+  <si>
+    <t>D584V</t>
+  </si>
+  <si>
+    <t>P527H</t>
+  </si>
+  <si>
+    <t>G625R</t>
+  </si>
+  <si>
+    <t>K438N</t>
+  </si>
+  <si>
+    <t>G449A</t>
+  </si>
+  <si>
+    <t>T508N</t>
+  </si>
+  <si>
+    <t>Y511H</t>
+  </si>
+  <si>
+    <t>S577L</t>
+  </si>
+  <si>
+    <t>A582V</t>
+  </si>
+  <si>
+    <t>N585K</t>
+  </si>
+  <si>
+    <t>Q613E</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -167,16 +286,41 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -184,15 +328,59 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -695,4 +883,320 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{723054C3-AE0C-004F-BA49-A7F8144721A5}">
+  <dimension ref="B1:C20"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="3" max="3" width="69.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B1" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="2" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B2" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="3" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B3" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B4" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="5" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B5" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="6" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B6" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="7" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B7" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="8" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B8" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="9" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B9" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="10" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B10" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="11" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B11" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="12" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B12" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="13" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B13" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="14" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B14" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="15" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B15" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="16" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B16" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B17" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="18" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B18" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="19" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B19" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="20" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B20" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15E8DA6C-79C8-EC42-A447-2DDC0D6B5EE4}">
+  <dimension ref="B1:H9"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B1" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="C1" s="6"/>
+      <c r="D1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="2" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B2" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="H2" s="8" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="3" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B3" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="4" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B4" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="5" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B5" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="H5" s="8" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="6" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B6" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="H6" s="8" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="7" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B7" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="8" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B8" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="H8" s="8" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="9" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="H9" s="8" t="s">
+        <v>77</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B1:C1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>